<commit_message>
features, changes, fix bugs, etc
</commit_message>
<xml_diff>
--- a/Template_Bulk_Challenges.xlsx
+++ b/Template_Bulk_Challenges.xlsx
@@ -3,8 +3,8 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Instructions" sheetId="1" r:id="rId1"/>
-    <sheet name="Challenges" sheetId="2" r:id="rId2"/>
+    <sheet name="Data" sheetId="1" r:id="rId1"/>
+    <sheet name="Instructions" sheetId="2" r:id="rId2"/>
   </sheets>
 </workbook>
 </file>
@@ -65,9 +65,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -399,195 +398,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A34"/>
-  <cols>
-    <col min="1" max="1" width="100.83203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>📋 INSTRUCCIONES - Bulk Upload de Challenges</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>COLUMNAS REQUERIDAS (obligatorias):</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v xml:space="preserve">  • Date            → Fecha en formato YYYY-MM-DD (ej: 2026-04-01). NO usar formato corto</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v xml:space="preserve">  • Title           → Nombre del challenge</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v xml:space="preserve">  • Description     → Descripción del challenge</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v xml:space="preserve">  • Type            → Tipo. SOLO 2 valores permitidos: Audio o MultipleChoice</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>COLUMNAS ADICIONALES PARA MultipleChoice (obligatorias si Type = MultipleChoice):</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v xml:space="preserve">  • Question        → Texto de la pregunta</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v xml:space="preserve">  • Options         → Opciones separadas por coma SIN espacios después de la coma</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v xml:space="preserve">                       Ejemplo correcto:   Hallo,Have,Hi</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v xml:space="preserve">                       Ejemplo INCORRECTO: Hallo, Have, Hi</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v xml:space="preserve">  • CorrectAnswer   → Número de la opción correcta (1, 2 o 3)</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <v xml:space="preserve">                       1 = primera opción, 2 = segunda, 3 = tercera</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="str">
-        <v>⚠️  REGLAS IMPORTANTES:</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="str">
-        <v xml:space="preserve">  1. NO se permiten fechas pasadas</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="str">
-        <v xml:space="preserve">  2. Máximo 30 challenges por carga</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="str">
-        <v xml:space="preserve">  3. Solo 1 challenge por día (no se pueden repetir fechas)</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="str">
-        <v xml:space="preserve">  4. Para challenges tipo Audio: solo llenar Date, Title, Description, Type</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="str">
-        <v xml:space="preserve">     Las columnas Question, Options, CorrectAnswer se dejan VACÍAS</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="str">
-        <v xml:space="preserve">  5. Para challenges tipo MultipleChoice: un challenge puede tener MÚLTIPLES preguntas</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="str">
-        <v xml:space="preserve">     Cada pregunta va en una fila separada, repitiendo Date, Title, Description, Type</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="str">
-        <v xml:space="preserve">     (ver ejemplo en la hoja 'Challenges')</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="str">
-        <v xml:space="preserve">  6. Las fechas DEBEN estar en formato YYYY-MM-DD</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="str">
-        <v xml:space="preserve">     Para que Excel no cambie el formato, seleccionar la columna Date y cambiar</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="str">
-        <v xml:space="preserve">     formato de celda a 'Texto' ANTES de escribir las fechas</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="str">
-        <v xml:space="preserve">  7. Type DEBE ser exactamente 'Audio' o 'MultipleChoice' (respetando mayúsculas)</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="str">
-        <v>💡 TIP: Ver los ejemplos en la hoja 'Challenges' →</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="str">
-        <v xml:space="preserve">   - Las filas 2-3: Challenge tipo Audio (solo 1 fila por challenge)</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="str">
-        <v xml:space="preserve">   - Las filas 4-8: Challenge tipo MultipleChoice con 5 preguntas (5 filas, misma fecha+título)</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="str">
-        <v xml:space="preserve">   - Las filas 9-11: Otro MultipleChoice con 3 preguntas</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A34"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G11"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
-    <col min="2" max="2" width="24.83203125" customWidth="1"/>
-    <col min="3" max="3" width="30.83203125" customWidth="1"/>
+    <col min="2" max="2" width="28.83203125" customWidth="1"/>
+    <col min="3" max="3" width="55.83203125" customWidth="1"/>
     <col min="4" max="4" width="16.83203125" customWidth="1"/>
     <col min="5" max="5" width="55.83203125" customWidth="1"/>
     <col min="6" max="6" width="30.83203125" customWidth="1"/>
@@ -618,14 +433,14 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="str">
+      <c r="A2" t="str">
         <v>2026-04-01</v>
       </c>
       <c r="B2" t="str">
         <v>Pronunciation Practice</v>
       </c>
       <c r="C2" t="str">
-        <v>Listen and repeat common business phrases</v>
+        <v>Listen and repeat common business phrases.</v>
       </c>
       <c r="D2" t="str">
         <v>Audio</v>
@@ -641,14 +456,14 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="str">
+      <c r="A3" t="str">
         <v>2026-04-02</v>
       </c>
       <c r="B3" t="str">
         <v>Listening Comprehension</v>
       </c>
       <c r="C3" t="str">
-        <v>Listen to a short conversation and answer</v>
+        <v>Listen to a short conversation and answer the questions.</v>
       </c>
       <c r="D3" t="str">
         <v>Audio</v>
@@ -664,7 +479,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="str">
+      <c r="A4" t="str">
         <v>2026-04-03</v>
       </c>
       <c r="B4" t="str">
@@ -682,12 +497,12 @@
       <c r="F4" t="str">
         <v>Hallo,Have,Hi</v>
       </c>
-      <c r="G4">
+      <c r="G4" t="str">
         <v>3</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="str">
+      <c r="A5" t="str">
         <v>2026-04-03</v>
       </c>
       <c r="B5" t="str">
@@ -705,12 +520,12 @@
       <c r="F5" t="str">
         <v>Hello,Good,Hi</v>
       </c>
-      <c r="G5">
+      <c r="G5" t="str">
         <v>2</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="str">
+      <c r="A6" t="str">
         <v>2026-04-03</v>
       </c>
       <c r="B6" t="str">
@@ -728,12 +543,12 @@
       <c r="F6" t="str">
         <v>a nice day,one,great</v>
       </c>
-      <c r="G6">
+      <c r="G6" t="str">
         <v>1</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="str">
+      <c r="A7" t="str">
         <v>2026-04-03</v>
       </c>
       <c r="B7" t="str">
@@ -751,12 +566,12 @@
       <c r="F7" t="str">
         <v>again,day,soon</v>
       </c>
-      <c r="G7">
+      <c r="G7" t="str">
         <v>3</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="str">
+      <c r="A8" t="str">
         <v>2026-04-03</v>
       </c>
       <c r="B8" t="str">
@@ -774,12 +589,12 @@
       <c r="F8" t="str">
         <v>Hello,Hey,Good day</v>
       </c>
-      <c r="G8">
+      <c r="G8" t="str">
         <v>2</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="str">
+      <c r="A9" t="str">
         <v>2026-04-04</v>
       </c>
       <c r="B9" t="str">
@@ -797,12 +612,12 @@
       <c r="F9" t="str">
         <v>Are,Am,Is</v>
       </c>
-      <c r="G9">
+      <c r="G9" t="str">
         <v>1</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="str">
+      <c r="A10" t="str">
         <v>2026-04-04</v>
       </c>
       <c r="B10" t="str">
@@ -815,17 +630,17 @@
         <v>MultipleChoice</v>
       </c>
       <c r="E10" t="str">
-        <v>Yes, I_______.</v>
+        <v>Yes, I _______.</v>
       </c>
       <c r="F10" t="str">
         <v>are,am,is</v>
       </c>
-      <c r="G10">
+      <c r="G10" t="str">
         <v>2</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="str">
+      <c r="A11" t="str">
         <v>2026-04-04</v>
       </c>
       <c r="B11" t="str">
@@ -843,7 +658,7 @@
       <c r="F11" t="str">
         <v>aren't,isn't,am not</v>
       </c>
-      <c r="G11">
+      <c r="G11" t="str">
         <v>3</v>
       </c>
     </row>
@@ -852,4 +667,245 @@
     <ignoredError numberStoredAsText="1" sqref="A1:G11"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D33"/>
+  <cols>
+    <col min="1" max="1" width="50.83203125" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
+    <col min="3" max="3" width="70.83203125" customWidth="1"/>
+    <col min="4" max="4" width="30.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>📋 BULK UPLOAD CHALLENGES — Instructions</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>REQUIRED COLUMNS</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Column</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Required</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Description</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Example</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Date</v>
+      </c>
+      <c r="B5" t="str">
+        <v>✅ Yes</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Challenge date. Supports: YYYY-MM-DD, DD-MM-YYYY, DD/MM/YYYY, or Excel serial dates. Only future dates allowed. Only ONE challenge per date.</v>
+      </c>
+      <c r="D5" t="str">
+        <v>2026-04-01</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Title</v>
+      </c>
+      <c r="B6" t="str">
+        <v>✅ Yes</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Title of the challenge.</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Grammar Quiz</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Description</v>
+      </c>
+      <c r="B7" t="str">
+        <v>✅ Yes</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Instructions or context for the challenge.</v>
+      </c>
+      <c r="D7" t="str">
+        <v>A1, Class 1: Greetings</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Type</v>
+      </c>
+      <c r="B8" t="str">
+        <v>✅ Yes</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Challenge type. Must be either: Audio or MultipleChoice.</v>
+      </c>
+      <c r="D8" t="str">
+        <v>MultipleChoice</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>MULTIPLE CHOICE COLUMNS (required when Type = MultipleChoice)</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Column</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Required</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Description</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Example</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Question</v>
+      </c>
+      <c r="B12" t="str">
+        <v>For MC</v>
+      </c>
+      <c r="C12" t="str">
+        <v>The question text. Use _____ as blank placeholder.</v>
+      </c>
+      <c r="D12" t="str">
+        <v>(Goodbye) Talk to you ______.</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Options</v>
+      </c>
+      <c r="B13" t="str">
+        <v>For MC</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Answer options separated by commas (no spaces around commas).</v>
+      </c>
+      <c r="D13" t="str">
+        <v>again,day,soon</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>CorrectAnswer</v>
+      </c>
+      <c r="B14" t="str">
+        <v>For MC</v>
+      </c>
+      <c r="C14" t="str">
+        <v>The number (1-based index) of the correct option from the Options list.</v>
+      </c>
+      <c r="D14" t="str">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>MULTIPLE QUESTIONS PER CHALLENGE</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>To add multiple questions to a single MultipleChoice challenge, repeat the same Date + Title + Description + Type on multiple rows. Each row adds one question.</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>Example: 5 rows with Date=2026-04-03, Title='Grammar Quiz' → creates 1 challenge with 5 questions.</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>SKILL BUILDER / SKILL BUILDER LIVE VISIBILITY</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>⚠️ These are NOT columns in the Excel file.</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>After uploading and previewing the file, you will see two checkboxes in the upload modal:</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v xml:space="preserve">  ☑ Visible for Skill Builder — Makes ALL uploaded challenges visible for Skill Builder plan users.</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v xml:space="preserve">  ☑ Visible for Skill Builder Live — Makes ALL uploaded challenges visible for Skill Builder Live plan users.</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>Both default to unchecked (not visible). The setting applies to ALL challenges in the batch.</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>LIMITS &amp; RULES</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>• Maximum 30 challenges per upload batch.</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>• Only future dates allowed (no past dates).</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>• Only ONE challenge per date (no duplicate dates in the batch).</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>• Supported file formats: .xlsx, .xls</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>• Audio challenges: only Date, Title, Description, Type are required (leave Question/Options/CorrectAnswer empty).</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>• MultipleChoice challenges: Question, Options and CorrectAnswer are required for each question row.</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:D1"/>
+  </mergeCells>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:D33"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>